<commit_message>
feat(periapuranam): selective backup Day3 — 11 runners + tracker + final txt (day-03)
- Day3 11/11 (56 files 217 chunks $2.3045): Muruga 4f, Muzhu 4f, Pugazh 4f, Chithaththaich 5f, Dhandi 5f, Perumizhalai 5f, Rudhra 5f, Eanati 6f, Manakkanchara 6f, Mara 6f, Viran Mindar 6f — all Chapter 04/05/06 no ==== finish:stop
- Viran Mindar fix: re-translated Chapter05 loop 1482x Thirumoolattanam (42k->11k) + removed stray Chapter 8 (94,947->62,819), rebuilt bilingual 234,598
- tracker periapuranam/day_wise_plan.xlsx Day3 + DayWise_Plan + Anomalies (Viran FIXED) updated
- template fix periapuranam/templates/run_nayanar_template.py payload_en max_tokens 12000->30000 applied to all 46 run_*.py (prevents truncation >40K Tamil)
- final outputs only: periapuranam/output/day-03/*/tamil_real/*_tamil.txt + /*_english.txt + /*_bilingual.txt (33 txt, 81 files total)
- ignore audio + chunk txt via .gitignore (output/**/audio/, *_chunk*.txt); folder structure preserved for later merge
</commit_message>
<xml_diff>
--- a/periapuranam/day_wise_plan.xlsx
+++ b/periapuranam/day_wise_plan.xlsx
@@ -41,7 +41,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="13">
     <font>
       <name val="Calibri"/>
@@ -116,7 +118,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -183,6 +185,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFE699"/>
         <bgColor rgb="00FFE699"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -270,7 +278,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -362,6 +370,21 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -966,16 +989,34 @@
           <t>$1.89</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr"/>
-      <c r="K4" s="5" t="inlineStr"/>
-      <c r="L4" s="5" t="inlineStr"/>
-      <c r="M4" s="5" t="inlineStr"/>
+      <c r="J4" s="36" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>56/56</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>~5.2h seq (217 chunks) + 11 translate</t>
+        </is>
+      </c>
+      <c r="M4" s="5" t="n">
+        <v>2.30449</v>
+      </c>
       <c r="N4" s="4" t="inlineStr">
         <is>
-          <t>11 stories Medium batch</t>
-        </is>
-      </c>
-      <c r="O4" s="2" t="inlineStr"/>
+          <t>11/11 PASS Chapter 4/5/6=ok no ==== finish:stop; viran_mindar Chapter05 loop fixed 42k-&gt;11k + removed stray Chapter 8; perumizhala resumed after network drop; verify Human Verified No pending spot-listen</t>
+        </is>
+      </c>
+      <c r="O4" s="37" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="52" customHeight="1">
       <c r="A5" s="2" t="n">
@@ -2183,7 +2224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2525,6 +2566,71 @@
       <c r="M5" s="35" t="inlineStr">
         <is>
           <t>INFO — keep flagged</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C6" s="39" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="D6" s="39" t="inlineStr">
+        <is>
+          <t>Viran Mindar Nayanar</t>
+        </is>
+      </c>
+      <c r="E6" s="39" t="inlineStr">
+        <is>
+          <t>Viran Mindar Nayanar</t>
+        </is>
+      </c>
+      <c r="F6" s="39" t="inlineStr">
+        <is>
+          <t>85,86,87,88,89,90 (Chapter 05 affected)</t>
+        </is>
+      </c>
+      <c r="G6" s="39" t="inlineStr">
+        <is>
+          <t>1SZcVJk3o46mKgshCnfTRpnHr9Zu96h7S et al. (seq 85-90; affected English Chapter 05)</t>
+        </is>
+      </c>
+      <c r="H6" s="39" t="inlineStr">
+        <is>
+          <t>viran_mindar_nayanar</t>
+        </is>
+      </c>
+      <c r="I6" s="39" t="inlineStr">
+        <is>
+          <t>periapuranam/output/day-03/viran_mindar_nayanar/viran_mindar_nayanar_english.txt</t>
+        </is>
+      </c>
+      <c r="J6" s="39" t="inlineStr">
+        <is>
+          <t>TRANSLATION HALLUCINATION + stray header</t>
+        </is>
+      </c>
+      <c r="K6" s="39" t="inlineStr">
+        <is>
+          <t>English Chapter 05 returned 42,594 chars with 1482x "Thirumoolattanam" / 1479x "in Thirumoolattanam," loop (vs Tamil 11,483). Also stray "Chapter 8, Religion..." block (1,111 chars) between Chapter 02 and 03. Story length inflated 94,947 vs correct 62,819. Classic Gemini 2.5-flash repetition loop.</t>
+        </is>
+      </c>
+      <c r="L6" s="39" t="inlineStr">
+        <is>
+          <t>Fixed 2026-09-14: Re-translated Tamil Chapter 05 alone (temp 0.3, 15k tokens) -&gt; 11,573 chars 1x Thirumoolattanam; removed stray Chapter 8 block; rebuilt english (62,819) + bilingual (234,598) + meta fix note. Verified 6ch, no ====, finish:stop. Keep for batch anomaly review in end.</t>
+        </is>
+      </c>
+      <c r="M6" s="40" t="inlineStr">
+        <is>
+          <t>FIXED 2026-09-14 - keep flagged for final review</t>
         </is>
       </c>
     </row>
@@ -5721,26 +5827,44 @@
           <t>muruga_nayanar</t>
         </is>
       </c>
-      <c r="I3" s="23" t="inlineStr">
-        <is>
-          <t>To be done</t>
-        </is>
-      </c>
-      <c r="J3" s="21" t="inlineStr"/>
-      <c r="K3" s="21" t="inlineStr"/>
-      <c r="L3" s="22" t="inlineStr"/>
-      <c r="M3" s="22" t="inlineStr"/>
-      <c r="N3" s="22" t="inlineStr"/>
+      <c r="I3" s="38" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J3" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="K3" s="21" t="n">
+        <v>16</v>
+      </c>
+      <c r="L3" s="22" t="n">
+        <v>0.1184</v>
+      </c>
+      <c r="M3" s="22" t="n">
+        <v>0.03379</v>
+      </c>
+      <c r="N3" s="22" t="n">
+        <v>0.15219</v>
+      </c>
       <c r="O3" s="21" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P3" s="22" t="inlineStr"/>
-      <c r="Q3" s="22" t="inlineStr"/>
+      <c r="P3" s="22" t="inlineStr">
+        <is>
+          <t>0 retries, all chunks OK</t>
+        </is>
+      </c>
+      <c r="Q3" s="22" t="inlineStr">
+        <is>
+          <t>Tamil 44694 chars /122651 bytes 4ch no ====; English 49473 chars finish:stop; total $0.15219</t>
+        </is>
+      </c>
       <c r="R3" s="22" t="inlineStr">
         <is>
-          <t>periapuranam/output/muruga_nayanar/tamil_real/muruga_nayanar_tamil.txt ; muruga_nayanar_english.txt</t>
+          <t>periapuranam/output/day-03/muruga_nayanar/tamil_real/muruga_nayanar_tamil.txt ; muruga_nayanar_english.txt</t>
         </is>
       </c>
     </row>
@@ -5779,26 +5903,44 @@
           <t>muzhu_neeru_poosiya_munivar</t>
         </is>
       </c>
-      <c r="I4" s="23" t="inlineStr">
-        <is>
-          <t>To be done</t>
-        </is>
-      </c>
-      <c r="J4" s="21" t="inlineStr"/>
-      <c r="K4" s="21" t="inlineStr"/>
-      <c r="L4" s="22" t="inlineStr"/>
-      <c r="M4" s="22" t="inlineStr"/>
-      <c r="N4" s="22" t="inlineStr"/>
+      <c r="I4" s="38" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J4" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="K4" s="21" t="n">
+        <v>15</v>
+      </c>
+      <c r="L4" s="22" t="n">
+        <v>0.12906</v>
+      </c>
+      <c r="M4" s="22" t="n">
+        <v>0.0377</v>
+      </c>
+      <c r="N4" s="22" t="n">
+        <v>0.16676</v>
+      </c>
       <c r="O4" s="21" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P4" s="22" t="inlineStr"/>
-      <c r="Q4" s="22" t="inlineStr"/>
+      <c r="P4" s="22" t="inlineStr">
+        <is>
+          <t>0 retries, all chunks OK</t>
+        </is>
+      </c>
+      <c r="Q4" s="22" t="inlineStr">
+        <is>
+          <t>Tamil 50653 chars /138556 bytes 4ch no ====; English 54429 chars finish:stop; total $0.16676</t>
+        </is>
+      </c>
       <c r="R4" s="22" t="inlineStr">
         <is>
-          <t>periapuranam/output/muzhu_neeru_poosiya_munivar/tamil_real/muzhu_neeru_poosiya_munivar_tamil.txt ; muzhu_neeru_poosiya_munivar_english.txt</t>
+          <t>periapuranam/output/day-03/muzhu_neeru_poosiya_munivar/tamil_real/muzhu_neeru_poosiya_munivar_tamil.txt ; muzhu_neeru_poosiya_munivar_english.txt</t>
         </is>
       </c>
     </row>
@@ -5837,26 +5979,44 @@
           <t>pugazh_chozha_nayanar</t>
         </is>
       </c>
-      <c r="I5" s="23" t="inlineStr">
-        <is>
-          <t>To be done</t>
-        </is>
-      </c>
-      <c r="J5" s="21" t="inlineStr"/>
-      <c r="K5" s="21" t="inlineStr"/>
-      <c r="L5" s="22" t="inlineStr"/>
-      <c r="M5" s="22" t="inlineStr"/>
-      <c r="N5" s="22" t="inlineStr"/>
+      <c r="I5" s="38" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J5" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="K5" s="21" t="n">
+        <v>14</v>
+      </c>
+      <c r="L5" s="22" t="n">
+        <v>0.10649</v>
+      </c>
+      <c r="M5" s="22" t="n">
+        <v>0.02946</v>
+      </c>
+      <c r="N5" s="22" t="n">
+        <v>0.13595</v>
+      </c>
       <c r="O5" s="21" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P5" s="22" t="inlineStr"/>
-      <c r="Q5" s="22" t="inlineStr"/>
+      <c r="P5" s="22" t="inlineStr">
+        <is>
+          <t>0 retries, all chunks OK</t>
+        </is>
+      </c>
+      <c r="Q5" s="22" t="inlineStr">
+        <is>
+          <t>Tamil 41532 chars /112724 bytes 4ch no ====; English 41532 chars finish:stop; total $0.13595</t>
+        </is>
+      </c>
       <c r="R5" s="22" t="inlineStr">
         <is>
-          <t>periapuranam/output/pugazh_chozha_nayanar/tamil_real/pugazh_chozha_nayanar_tamil.txt ; pugazh_chozha_nayanar_english.txt</t>
+          <t>periapuranam/output/day-03/pugazh_chozha_nayanar/tamil_real/pugazh_chozha_nayanar_tamil.txt ; pugazh_chozha_nayanar_english.txt</t>
         </is>
       </c>
     </row>
@@ -5895,26 +6055,44 @@
           <t>chithaththaich_sivan_pale_vaiththar</t>
         </is>
       </c>
-      <c r="I6" s="23" t="inlineStr">
-        <is>
-          <t>To be done</t>
-        </is>
-      </c>
-      <c r="J6" s="21" t="inlineStr"/>
-      <c r="K6" s="21" t="inlineStr"/>
-      <c r="L6" s="22" t="inlineStr"/>
-      <c r="M6" s="22" t="inlineStr"/>
-      <c r="N6" s="22" t="inlineStr"/>
+      <c r="I6" s="38" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J6" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="K6" s="21" t="n">
+        <v>20</v>
+      </c>
+      <c r="L6" s="22" t="n">
+        <v>0.17726</v>
+      </c>
+      <c r="M6" s="22" t="n">
+        <v>0.0491</v>
+      </c>
+      <c r="N6" s="22" t="n">
+        <v>0.22636</v>
+      </c>
       <c r="O6" s="21" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P6" s="22" t="inlineStr"/>
-      <c r="Q6" s="22" t="inlineStr"/>
+      <c r="P6" s="22" t="inlineStr">
+        <is>
+          <t>0 retries, all chunks OK</t>
+        </is>
+      </c>
+      <c r="Q6" s="22" t="inlineStr">
+        <is>
+          <t>Tamil 65514 chars /178569 bytes 5ch no ====; English 74889 chars finish:stop; total $0.22636</t>
+        </is>
+      </c>
       <c r="R6" s="22" t="inlineStr">
         <is>
-          <t>periapuranam/output/chithaththaich_sivan_pale_vaiththar/tamil_real/chithaththaich_sivan_pale_vaiththar_tamil.txt ; chithaththaich_sivan_pale_vaiththar_english.txt</t>
+          <t>periapuranam/output/day-03/chithaththaich_sivan_pale_vaiththar/tamil_real/chithaththaich_sivan_pale_vaiththar_tamil.txt ; chithaththaich_sivan_pale_vaiththar_english.txt</t>
         </is>
       </c>
     </row>
@@ -5953,26 +6131,44 @@
           <t>dhandi_adigal_nayanar</t>
         </is>
       </c>
-      <c r="I7" s="23" t="inlineStr">
-        <is>
-          <t>To be done</t>
-        </is>
-      </c>
-      <c r="J7" s="21" t="inlineStr"/>
-      <c r="K7" s="21" t="inlineStr"/>
-      <c r="L7" s="22" t="inlineStr"/>
-      <c r="M7" s="22" t="inlineStr"/>
-      <c r="N7" s="22" t="inlineStr"/>
+      <c r="I7" s="38" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J7" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="K7" s="21" t="n">
+        <v>24</v>
+      </c>
+      <c r="L7" s="22" t="n">
+        <v>0.21459</v>
+      </c>
+      <c r="M7" s="22" t="n">
+        <v>0.06136</v>
+      </c>
+      <c r="N7" s="22" t="n">
+        <v>0.27595</v>
+      </c>
       <c r="O7" s="21" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P7" s="22" t="inlineStr"/>
-      <c r="Q7" s="22" t="inlineStr"/>
+      <c r="P7" s="22" t="inlineStr">
+        <is>
+          <t>0 retries, all chunks OK</t>
+        </is>
+      </c>
+      <c r="Q7" s="22" t="inlineStr">
+        <is>
+          <t>Tamil 80590 chars /220757 bytes 5ch no ====; English 88826 chars finish:stop; total $0.27595</t>
+        </is>
+      </c>
       <c r="R7" s="22" t="inlineStr">
         <is>
-          <t>periapuranam/output/dhandi_adigal_nayanar/tamil_real/dhandi_adigal_nayanar_tamil.txt ; dhandi_adigal_nayanar_english.txt</t>
+          <t>periapuranam/output/day-03/dhandi_adigal_nayanar/tamil_real/dhandi_adigal_nayanar_tamil.txt ; dhandi_adigal_nayanar_english.txt</t>
         </is>
       </c>
     </row>
@@ -6011,26 +6207,44 @@
           <t>perumizhalaikurumba_nayanar</t>
         </is>
       </c>
-      <c r="I8" s="23" t="inlineStr">
-        <is>
-          <t>To be done</t>
-        </is>
-      </c>
-      <c r="J8" s="21" t="inlineStr"/>
-      <c r="K8" s="21" t="inlineStr"/>
-      <c r="L8" s="22" t="inlineStr"/>
-      <c r="M8" s="22" t="inlineStr"/>
-      <c r="N8" s="22" t="inlineStr"/>
+      <c r="I8" s="38" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J8" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="K8" s="21" t="n">
+        <v>18</v>
+      </c>
+      <c r="L8" s="22" t="n">
+        <v>0.15865</v>
+      </c>
+      <c r="M8" s="22" t="n">
+        <v>0.04071</v>
+      </c>
+      <c r="N8" s="22" t="n">
+        <v>0.19936</v>
+      </c>
       <c r="O8" s="21" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P8" s="22" t="inlineStr"/>
-      <c r="Q8" s="22" t="inlineStr"/>
+      <c r="P8" s="22" t="inlineStr">
+        <is>
+          <t>1 retry ConnectionReset 10054 chunk01 auto-recovered; resumed from 483 partial</t>
+        </is>
+      </c>
+      <c r="Q8" s="22" t="inlineStr">
+        <is>
+          <t>Tamil 58220 chars /160077 bytes 5ch no ====; English 58138 chars finish:stop; total $0.19936</t>
+        </is>
+      </c>
       <c r="R8" s="22" t="inlineStr">
         <is>
-          <t>periapuranam/output/perumizhalaikurumba_nayanar/tamil_real/perumizhalaikurumba_nayanar_tamil.txt ; perumizhalaikurumba_nayanar_english.txt</t>
+          <t>periapuranam/output/day-03/perumizhalaikurumba_nayanar/tamil_real/perumizhalaikurumba_nayanar_tamil.txt ; perumizhalaikurumba_nayanar_english.txt</t>
         </is>
       </c>
     </row>
@@ -6069,26 +6283,44 @@
           <t>rudhra_pasupadhi_nayanar</t>
         </is>
       </c>
-      <c r="I9" s="23" t="inlineStr">
-        <is>
-          <t>To be done</t>
-        </is>
-      </c>
-      <c r="J9" s="21" t="inlineStr"/>
-      <c r="K9" s="21" t="inlineStr"/>
-      <c r="L9" s="22" t="inlineStr"/>
-      <c r="M9" s="22" t="inlineStr"/>
-      <c r="N9" s="22" t="inlineStr"/>
+      <c r="I9" s="38" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J9" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="K9" s="21" t="n">
+        <v>18</v>
+      </c>
+      <c r="L9" s="22" t="n">
+        <v>0.13727</v>
+      </c>
+      <c r="M9" s="22" t="n">
+        <v>0.03606</v>
+      </c>
+      <c r="N9" s="22" t="n">
+        <v>0.17333</v>
+      </c>
       <c r="O9" s="21" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P9" s="22" t="inlineStr"/>
-      <c r="Q9" s="22" t="inlineStr"/>
+      <c r="P9" s="22" t="inlineStr">
+        <is>
+          <t>0 retries, all chunks OK</t>
+        </is>
+      </c>
+      <c r="Q9" s="22" t="inlineStr">
+        <is>
+          <t>Tamil 49083 chars /134438 bytes 5ch no ====; English 51607 chars finish:stop; total $0.17333</t>
+        </is>
+      </c>
       <c r="R9" s="22" t="inlineStr">
         <is>
-          <t>periapuranam/output/rudhra_pasupadhi_nayanar/tamil_real/rudhra_pasupadhi_nayanar_tamil.txt ; rudhra_pasupadhi_nayanar_english.txt</t>
+          <t>periapuranam/output/day-03/rudhra_pasupadhi_nayanar/tamil_real/rudhra_pasupadhi_nayanar_tamil.txt ; rudhra_pasupadhi_nayanar_english.txt</t>
         </is>
       </c>
     </row>
@@ -6127,26 +6359,44 @@
           <t>eanati_nathar_nayanar</t>
         </is>
       </c>
-      <c r="I10" s="23" t="inlineStr">
-        <is>
-          <t>To be done</t>
-        </is>
-      </c>
-      <c r="J10" s="21" t="inlineStr"/>
-      <c r="K10" s="21" t="inlineStr"/>
-      <c r="L10" s="22" t="inlineStr"/>
-      <c r="M10" s="22" t="inlineStr"/>
-      <c r="N10" s="22" t="inlineStr"/>
+      <c r="I10" s="38" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J10" s="21" t="n">
+        <v>6</v>
+      </c>
+      <c r="K10" s="21" t="n">
+        <v>24</v>
+      </c>
+      <c r="L10" s="22" t="n">
+        <v>0.2021</v>
+      </c>
+      <c r="M10" s="22" t="n">
+        <v>0.04804</v>
+      </c>
+      <c r="N10" s="22" t="n">
+        <v>0.25014</v>
+      </c>
       <c r="O10" s="21" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P10" s="22" t="inlineStr"/>
-      <c r="Q10" s="22" t="inlineStr"/>
+      <c r="P10" s="22" t="inlineStr">
+        <is>
+          <t>0 retries, all chunks OK</t>
+        </is>
+      </c>
+      <c r="Q10" s="22" t="inlineStr">
+        <is>
+          <t>Tamil 71655 chars /195984 bytes 6ch no ====; English 71943 chars finish:stop; total $0.25014</t>
+        </is>
+      </c>
       <c r="R10" s="22" t="inlineStr">
         <is>
-          <t>periapuranam/output/eanati_nathar_nayanar/tamil_real/eanati_nathar_nayanar_tamil.txt ; eanati_nathar_nayanar_english.txt</t>
+          <t>periapuranam/output/day-03/eanati_nathar_nayanar/tamil_real/eanati_nathar_nayanar_tamil.txt ; eanati_nathar_nayanar_english.txt</t>
         </is>
       </c>
     </row>
@@ -6185,26 +6435,44 @@
           <t>manakkanchara_nayanar</t>
         </is>
       </c>
-      <c r="I11" s="23" t="inlineStr">
-        <is>
-          <t>To be done</t>
-        </is>
-      </c>
-      <c r="J11" s="21" t="inlineStr"/>
-      <c r="K11" s="21" t="inlineStr"/>
-      <c r="L11" s="22" t="inlineStr"/>
-      <c r="M11" s="22" t="inlineStr"/>
-      <c r="N11" s="22" t="inlineStr"/>
+      <c r="I11" s="38" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J11" s="21" t="n">
+        <v>6</v>
+      </c>
+      <c r="K11" s="21" t="n">
+        <v>22</v>
+      </c>
+      <c r="L11" s="22" t="n">
+        <v>0.19038</v>
+      </c>
+      <c r="M11" s="22" t="n">
+        <v>0.04927</v>
+      </c>
+      <c r="N11" s="22" t="n">
+        <v>0.23965</v>
+      </c>
       <c r="O11" s="21" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P11" s="22" t="inlineStr"/>
-      <c r="Q11" s="22" t="inlineStr"/>
+      <c r="P11" s="22" t="inlineStr">
+        <is>
+          <t>0 retries, all chunks OK</t>
+        </is>
+      </c>
+      <c r="Q11" s="22" t="inlineStr">
+        <is>
+          <t>Tamil 67618 chars /185695 bytes 6ch no ====; English 70503 chars finish:stop; total $0.23965</t>
+        </is>
+      </c>
       <c r="R11" s="22" t="inlineStr">
         <is>
-          <t>periapuranam/output/manakkanchara_nayanar/tamil_real/manakkanchara_nayanar_tamil.txt ; manakkanchara_nayanar_english.txt</t>
+          <t>periapuranam/output/day-03/manakkanchara_nayanar/tamil_real/manakkanchara_nayanar_tamil.txt ; manakkanchara_nayanar_english.txt</t>
         </is>
       </c>
     </row>
@@ -6243,26 +6511,44 @@
           <t>mara_nayanar</t>
         </is>
       </c>
-      <c r="I12" s="23" t="inlineStr">
-        <is>
-          <t>To be done</t>
-        </is>
-      </c>
-      <c r="J12" s="21" t="inlineStr"/>
-      <c r="K12" s="21" t="inlineStr"/>
-      <c r="L12" s="22" t="inlineStr"/>
-      <c r="M12" s="22" t="inlineStr"/>
-      <c r="N12" s="22" t="inlineStr"/>
+      <c r="I12" s="38" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J12" s="21" t="n">
+        <v>6</v>
+      </c>
+      <c r="K12" s="21" t="n">
+        <v>24</v>
+      </c>
+      <c r="L12" s="22" t="n">
+        <v>0.19646</v>
+      </c>
+      <c r="M12" s="22" t="n">
+        <v>0.04678</v>
+      </c>
+      <c r="N12" s="22" t="n">
+        <v>0.24324</v>
+      </c>
       <c r="O12" s="21" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P12" s="22" t="inlineStr"/>
-      <c r="Q12" s="22" t="inlineStr"/>
+      <c r="P12" s="22" t="inlineStr">
+        <is>
+          <t>0 retries, all chunks OK</t>
+        </is>
+      </c>
+      <c r="Q12" s="22" t="inlineStr">
+        <is>
+          <t>Tamil 72124 chars /197919 bytes 6ch no ====; English 71030 chars finish:stop; total $0.24324</t>
+        </is>
+      </c>
       <c r="R12" s="22" t="inlineStr">
         <is>
-          <t>periapuranam/output/mara_nayanar/tamil_real/mara_nayanar_tamil.txt ; mara_nayanar_english.txt</t>
+          <t>periapuranam/output/day-03/mara_nayanar/tamil_real/mara_nayanar_tamil.txt ; mara_nayanar_english.txt</t>
         </is>
       </c>
     </row>
@@ -6301,26 +6587,44 @@
           <t>viran_mindar</t>
         </is>
       </c>
-      <c r="I13" s="23" t="inlineStr">
-        <is>
-          <t>To be done</t>
-        </is>
-      </c>
-      <c r="J13" s="21" t="inlineStr"/>
-      <c r="K13" s="21" t="inlineStr"/>
-      <c r="L13" s="22" t="inlineStr"/>
-      <c r="M13" s="22" t="inlineStr"/>
-      <c r="N13" s="22" t="inlineStr"/>
+      <c r="I13" s="38" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J13" s="21" t="n">
+        <v>6</v>
+      </c>
+      <c r="K13" s="21" t="n">
+        <v>22</v>
+      </c>
+      <c r="L13" s="22" t="n">
+        <v>0.17292</v>
+      </c>
+      <c r="M13" s="22" t="n">
+        <v>0.06864000000000001</v>
+      </c>
+      <c r="N13" s="22" t="n">
+        <v>0.24156</v>
+      </c>
       <c r="O13" s="21" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P13" s="22" t="inlineStr"/>
-      <c r="Q13" s="22" t="inlineStr"/>
+      <c r="P13" s="22" t="inlineStr">
+        <is>
+          <t>1 fix: Chapter05 1479x Thirumoolattanam loop re-translated</t>
+        </is>
+      </c>
+      <c r="Q13" s="22" t="inlineStr">
+        <is>
+          <t>Tamil 62406 chars /171695 bytes 6ch no ====; English 62819 chars finish:stop; total $0.24156 FIXED Chapter05 loop removed, stray Chapter 8 removed (94k-&gt;62k)</t>
+        </is>
+      </c>
       <c r="R13" s="22" t="inlineStr">
         <is>
-          <t>periapuranam/output/viran_mindar/tamil_real/viran_mindar_tamil.txt ; viran_mindar_english.txt</t>
+          <t>periapuranam/output/day-03/viran_mindar_nayanar/tamil_real/viran_mindar_nayanar_tamil.txt ; viran_mindar_nayanar_english.txt</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(periapuranam): Day5 3/6 3-parallel 38m wall 120ch + 524 fix + batch wrapper
Murthi 11F 43ch 129k/125k + Tiruneelanakkar 11F 35ch 100k/99k + Appoothi 12F 42ch 129k/120k all no ==== Chapter N==files 0 anomalies (524 30s 0->397c re-transcribed + re-translated). Budget fail-fast 402/403 -> sys.exit(2) patched 60 runners + template (was 3x retry 22c). Resume cached skip added. 3-parallel throttle 2.0s +30s stagger validated 38m wall vs 120m seq. Progress wrapper run_day05_batch.py with batch_progress.json meter for remaining Amar/Eri/Siruthonda 39F 136ch. Tracker DayWise Im Progress 34/73 1.2142.
</commit_message>
<xml_diff>
--- a/periapuranam/day_wise_plan.xlsx
+++ b/periapuranam/day_wise_plan.xlsx
@@ -41,8 +41,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -278,7 +279,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -385,6 +386,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -895,16 +905,34 @@
           <t>$0.71</t>
         </is>
       </c>
-      <c r="J2" s="5" t="inlineStr"/>
-      <c r="K2" s="5" t="inlineStr"/>
-      <c r="L2" s="5" t="inlineStr"/>
-      <c r="M2" s="5" t="inlineStr"/>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>21/21</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>86 chunks (21 translate)</t>
+        </is>
+      </c>
+      <c r="M2" s="41" t="n">
+        <v>0.9644</v>
+      </c>
       <c r="N2" s="4" t="inlineStr">
         <is>
-          <t>21 output folders in day-01/ — Verify Chapter 01=1, no ==== | FLAGGED: Poyyadiai illadha Nayanar (967) WRONG CONTENT (Kootruva duplicate) — flagged in Day 1 row14, await actual source</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="inlineStr"/>
+          <t>21/21 PASS Chapter 01=1 no ==== finish:stop; 1 flagged Poyyadiai WRONG (Kootruva dup) pending source</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="52" customHeight="1">
       <c r="A3" s="2" t="n">
@@ -942,16 +970,34 @@
           <t>$1.15</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr"/>
-      <c r="K3" s="5" t="inlineStr"/>
-      <c r="L3" s="5" t="inlineStr"/>
-      <c r="M3" s="5" t="inlineStr"/>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>14/14</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>123 chunks (14 translate)</t>
+        </is>
+      </c>
+      <c r="M3" s="41" t="n">
+        <v>1.3558</v>
+      </c>
       <c r="N3" s="4" t="inlineStr">
         <is>
-          <t>14 stories Thillai Vazh Anthanar 3 files -&gt; C01..03</t>
-        </is>
-      </c>
-      <c r="O3" s="2" t="inlineStr"/>
+          <t>14/14 PASS Chapter 02/03=ok no ====; 2 anomalies KazharChinga 41832 + Thillai 0-char deferred; AdhiBaththa INFO duplicate fid</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="52" customHeight="1">
       <c r="A4" s="2" t="n">
@@ -1004,7 +1050,7 @@
           <t>~5.2h seq (217 chunks) + 11 translate</t>
         </is>
       </c>
-      <c r="M4" s="5" t="n">
+      <c r="M4" s="41" t="n">
         <v>2.30449</v>
       </c>
       <c r="N4" s="4" t="inlineStr">
@@ -1051,23 +1097,27 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
+          <t>$1.88</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="K5" s="5" t="inlineStr">
         <is>
           <t>56/56</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="L5" s="5" t="inlineStr">
         <is>
           <t>223 chunks 2-workers + fixes</t>
         </is>
       </c>
-      <c r="L5" s="5" t="n">
+      <c r="M5" s="41" t="n">
         <v>2.3147</v>
       </c>
-      <c r="M5" s="5" t="inlineStr"/>
       <c r="N5" s="4" t="inlineStr">
         <is>
           <t>Day4 7/7 PASS Chapter N==files no ====; ThiruMoola/Tiru 0 anomalies dur-aware; Mei 083 fixed; Iyar HUGE fixed; Sak chunked translate</t>
@@ -1115,16 +1165,34 @@
           <t>$2.45</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr"/>
-      <c r="K6" s="5" t="inlineStr"/>
-      <c r="L6" s="5" t="inlineStr"/>
-      <c r="M6" s="5" t="inlineStr"/>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>34/73 (3/6 stories)</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>120ch 3-parallel 38m +524 fix</t>
+        </is>
+      </c>
+      <c r="M6" s="41" t="n">
+        <v>1.2142</v>
+      </c>
       <c r="N6" s="4" t="inlineStr">
         <is>
-          <t>6 stories Siruthonda 13 files</t>
-        </is>
-      </c>
-      <c r="O6" s="2" t="inlineStr"/>
+          <t>Murthi/Tiru/Appoothi DONE 0 anomalies (1 fixed), remaining Amar/Eri/Siruthonda 39F via batch wrapper</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="52" customHeight="1">
       <c r="A7" s="2" t="n">
@@ -7479,21 +7547,41 @@
       </c>
       <c r="I3" s="23" t="inlineStr">
         <is>
-          <t>To be done</t>
-        </is>
-      </c>
-      <c r="J3" s="21" t="inlineStr"/>
-      <c r="K3" s="21" t="inlineStr"/>
-      <c r="L3" s="22" t="inlineStr"/>
-      <c r="M3" s="22" t="inlineStr"/>
-      <c r="N3" s="22" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J3" s="21" t="inlineStr">
+        <is>
+          <t>11/11</t>
+        </is>
+      </c>
+      <c r="K3" s="42" t="n">
+        <v>43</v>
+      </c>
+      <c r="L3" s="43" t="n">
+        <v>0.3516</v>
+      </c>
+      <c r="M3" s="43" t="n">
+        <v>0.08450000000000001</v>
+      </c>
+      <c r="N3" s="43" t="n">
+        <v>0.4361</v>
+      </c>
       <c r="O3" s="21" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P3" s="22" t="inlineStr"/>
-      <c r="Q3" s="22" t="inlineStr"/>
+      <c r="P3" s="22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Q3" s="22" t="inlineStr">
+        <is>
+          <t>3-parallel 38m wall 0 anomalies 2103s no ==== Chapter 11/11</t>
+        </is>
+      </c>
       <c r="R3" s="22" t="inlineStr">
         <is>
           <t>periapuranam/output/murthi_nayanar/tamil_real/murthi_nayanar_tamil.txt ; murthi_nayanar_english.txt</t>
@@ -7537,21 +7625,41 @@
       </c>
       <c r="I4" s="23" t="inlineStr">
         <is>
-          <t>To be done</t>
-        </is>
-      </c>
-      <c r="J4" s="21" t="inlineStr"/>
-      <c r="K4" s="21" t="inlineStr"/>
-      <c r="L4" s="22" t="inlineStr"/>
-      <c r="M4" s="22" t="inlineStr"/>
-      <c r="N4" s="22" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J4" s="21" t="inlineStr">
+        <is>
+          <t>11/11</t>
+        </is>
+      </c>
+      <c r="K4" s="42" t="n">
+        <v>35</v>
+      </c>
+      <c r="L4" s="43" t="n">
+        <v>0.2778</v>
+      </c>
+      <c r="M4" s="43" t="n">
+        <v>0.0675</v>
+      </c>
+      <c r="N4" s="43" t="n">
+        <v>0.3453</v>
+      </c>
       <c r="O4" s="21" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P4" s="22" t="inlineStr"/>
-      <c r="Q4" s="22" t="inlineStr"/>
+      <c r="P4" s="22" t="inlineStr">
+        <is>
+          <t>1 re-transcribe 524/3 0-&gt;397c</t>
+        </is>
+      </c>
+      <c r="Q4" s="22" t="inlineStr">
+        <is>
+          <t>30s tail fixed 0 anomalies now 1799s no ====</t>
+        </is>
+      </c>
       <c r="R4" s="22" t="inlineStr">
         <is>
           <t>periapuranam/output/tiruneelanakkar_nayanar/tamil_real/tiruneelanakkar_nayanar_tamil.txt ; tiruneelanakkar_nayanar_english.txt</t>
@@ -7595,21 +7703,41 @@
       </c>
       <c r="I5" s="23" t="inlineStr">
         <is>
-          <t>To be done</t>
-        </is>
-      </c>
-      <c r="J5" s="21" t="inlineStr"/>
-      <c r="K5" s="21" t="inlineStr"/>
-      <c r="L5" s="22" t="inlineStr"/>
-      <c r="M5" s="22" t="inlineStr"/>
-      <c r="N5" s="22" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J5" s="21" t="inlineStr">
+        <is>
+          <t>12/12</t>
+        </is>
+      </c>
+      <c r="K5" s="42" t="n">
+        <v>42</v>
+      </c>
+      <c r="L5" s="43" t="n">
+        <v>0.3484</v>
+      </c>
+      <c r="M5" s="43" t="n">
+        <v>0.0844</v>
+      </c>
+      <c r="N5" s="43" t="n">
+        <v>0.4328</v>
+      </c>
       <c r="O5" s="21" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P5" s="22" t="inlineStr"/>
-      <c r="Q5" s="22" t="inlineStr"/>
+      <c r="P5" s="22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Q5" s="22" t="inlineStr">
+        <is>
+          <t>3-parallel 0 anomalies 2038s no ==== Chapter 12/12</t>
+        </is>
+      </c>
       <c r="R5" s="22" t="inlineStr">
         <is>
           <t>periapuranam/output/appoothi_adikal_nayanar/tamil_real/appoothi_adikal_nayanar_tamil.txt ; appoothi_adikal_nayanar_english.txt</t>

</xml_diff>

<commit_message>
feat(periapuranam): Day5 6/6 two-pass 73F 269ch + chunked English english_real
- Tamil Pass1 fix 4 chunks: 095 HUGE 43k->176c re-download 14.2M (ffmpeg 900s Invalid), 111 TINY 7->81c, 926 TINY 7->89c, 928 EMPTY 0->544c; stories 376K/417K/410K 13ch no ==== stop
- English Pass2 chunked 60K limit 3x3 english_real: amar 58857+48347+25003=132K, eri 52962+57487+44760=155K, siru 44444+55733+42806=142K stop 0 anomalies
- Meter event+heartbeat (POLL 30s HEARTBEAT 300s filesystem count, -u unbuffered, RESUME 38/136)
- Tracker DayWise 73/73 Done 269ch 2.42 Day5 sheet 6 rows + lessons-learnt.md
- Day6 queued 96F 336ch two-pass
</commit_message>
<xml_diff>
--- a/periapuranam/day_wise_plan.xlsx
+++ b/periapuranam/day_wise_plan.xlsx
@@ -1167,30 +1167,30 @@
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>34/73 (3/6 stories)</t>
+          <t>73/73 (6/6 stories)</t>
         </is>
       </c>
       <c r="L6" s="5" t="inlineStr">
         <is>
-          <t>120ch 3-parallel 38m +524 fix</t>
+          <t>269ch 3-parallel 38m + Tamil fix 4ch 4m + English chunked 9ch 10m (52m wall)</t>
         </is>
       </c>
       <c r="M6" s="41" t="n">
-        <v>1.2142</v>
+        <v>2.4193</v>
       </c>
       <c r="N6" s="4" t="inlineStr">
         <is>
-          <t>Murthi/Tiru/Appoothi DONE 0 anomalies (1 fixed), remaining Amar/Eri/Siruthonda 39F via batch wrapper</t>
+          <t>6/6 DONE 11+11+12+13+13+13 ch 43+35+42+48+53+48 no ==== Ch 11/11 12/12 13/13/13 fix 095 HUGE 43k-&gt;176c re-download +3 tails; English chunked 3x3 english_real stop</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -7781,24 +7781,44 @@
       </c>
       <c r="I6" s="23" t="inlineStr">
         <is>
-          <t>To be done</t>
-        </is>
-      </c>
-      <c r="J6" s="21" t="inlineStr"/>
-      <c r="K6" s="21" t="inlineStr"/>
-      <c r="L6" s="22" t="inlineStr"/>
-      <c r="M6" s="22" t="inlineStr"/>
-      <c r="N6" s="22" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J6" s="21" t="inlineStr">
+        <is>
+          <t>13/13</t>
+        </is>
+      </c>
+      <c r="K6" s="21" t="n">
+        <v>48</v>
+      </c>
+      <c r="L6" s="22" t="n">
+        <v>0.2747</v>
+      </c>
+      <c r="M6" s="22" t="n">
+        <v>0.0905</v>
+      </c>
+      <c r="N6" s="22" t="n">
+        <v>0.3652</v>
+      </c>
       <c r="O6" s="21" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P6" s="22" t="inlineStr"/>
-      <c r="Q6" s="22" t="inlineStr"/>
+      <c r="P6" s="22" t="inlineStr">
+        <is>
+          <t>1 fix 095 HUGE 43198-&gt;176c re-download 14.2M + chunk 43k-&gt;176c</t>
+        </is>
+      </c>
+      <c r="Q6" s="22" t="inlineStr">
+        <is>
+          <t>3-parallel then Tamil fix + English chunked 3/3 58857+48347+25003 english_real 0 anomalies</t>
+        </is>
+      </c>
       <c r="R6" s="22" t="inlineStr">
         <is>
-          <t>periapuranam/output/amar_niti_nayanar/tamil_real/amar_niti_nayanar_tamil.txt ; amar_niti_nayanar_english.txt</t>
+          <t>periapuranam/output/day-05/amar_niti_nayanar/tamil_real/amar_niti_nayanar_tamil.txt ; amar_niti_nayanar_english.txt ; english_real/3 chunks</t>
         </is>
       </c>
     </row>
@@ -7839,24 +7859,44 @@
       </c>
       <c r="I7" s="23" t="inlineStr">
         <is>
-          <t>To be done</t>
-        </is>
-      </c>
-      <c r="J7" s="21" t="inlineStr"/>
-      <c r="K7" s="21" t="inlineStr"/>
-      <c r="L7" s="22" t="inlineStr"/>
-      <c r="M7" s="22" t="inlineStr"/>
-      <c r="N7" s="22" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J7" s="21" t="inlineStr">
+        <is>
+          <t>13/13</t>
+        </is>
+      </c>
+      <c r="K7" s="21" t="n">
+        <v>53</v>
+      </c>
+      <c r="L7" s="22" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="M7" s="22" t="n">
+        <v>0.1054</v>
+      </c>
+      <c r="N7" s="22" t="n">
+        <v>0.4384</v>
+      </c>
       <c r="O7" s="21" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P7" s="22" t="inlineStr"/>
-      <c r="Q7" s="22" t="inlineStr"/>
+      <c r="P7" s="22" t="inlineStr">
+        <is>
+          <t>1 fix 111 TINY 7-&gt;81c</t>
+        </is>
+      </c>
+      <c r="Q7" s="22" t="inlineStr">
+        <is>
+          <t>English chunked 3/3 52962+57487+44760 0 anomalies</t>
+        </is>
+      </c>
       <c r="R7" s="22" t="inlineStr">
         <is>
-          <t>periapuranam/output/eri_pattha_nayanar/tamil_real/eri_pattha_nayanar_tamil.txt ; eri_pattha_nayanar_english.txt</t>
+          <t>periapuranam/output/day-05/eri_pattha_nayanar/tamil_real/eri_pattha_nayanar_tamil.txt ; eri_pattha_nayanar_english.txt ; english_real/3 chunks</t>
         </is>
       </c>
     </row>
@@ -7897,24 +7937,44 @@
       </c>
       <c r="I8" s="23" t="inlineStr">
         <is>
-          <t>To be done</t>
-        </is>
-      </c>
-      <c r="J8" s="21" t="inlineStr"/>
-      <c r="K8" s="21" t="inlineStr"/>
-      <c r="L8" s="22" t="inlineStr"/>
-      <c r="M8" s="22" t="inlineStr"/>
-      <c r="N8" s="22" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J8" s="21" t="inlineStr">
+        <is>
+          <t>13/13</t>
+        </is>
+      </c>
+      <c r="K8" s="21" t="n">
+        <v>48</v>
+      </c>
+      <c r="L8" s="22" t="n">
+        <v>0.3046</v>
+      </c>
+      <c r="M8" s="22" t="n">
+        <v>0.0969</v>
+      </c>
+      <c r="N8" s="22" t="n">
+        <v>0.4015</v>
+      </c>
       <c r="O8" s="21" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P8" s="22" t="inlineStr"/>
-      <c r="Q8" s="22" t="inlineStr"/>
+      <c r="P8" s="22" t="inlineStr">
+        <is>
+          <t>2 fix 926 TINY 7-&gt;89c + 928 EMPTY 0-&gt;544c</t>
+        </is>
+      </c>
+      <c r="Q8" s="22" t="inlineStr">
+        <is>
+          <t>English chunked 3/3 44444+55733+42806 0 anomalies</t>
+        </is>
+      </c>
       <c r="R8" s="22" t="inlineStr">
         <is>
-          <t>periapuranam/output/siruthonda_nayanar/tamil_real/siruthonda_nayanar_tamil.txt ; siruthonda_nayanar_english.txt</t>
+          <t>periapuranam/output/day-05/siruthonda_nayanar/tamil_real/siruthonda_nayanar_tamil.txt ; siruthonda_nayanar_english.txt ; english_real/3 chunks</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(periapuranam): Day6 4/4 96F 362ch heritage complete — Kazhar 28F 287K 6ch + Kannappa 32F 435K 9ch sequential 60K english_real, Tamil tails fixed 128/147, Day6 wall ~177m cost $3.84
</commit_message>
<xml_diff>
--- a/periapuranam/day_wise_plan.xlsx
+++ b/periapuranam/day_wise_plan.xlsx
@@ -1230,28 +1230,32 @@
           <t>$3.24</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr"/>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
-          <t>36/96 (2/4 stories)</t>
+          <t>96/96 (4/4 stories)</t>
         </is>
       </c>
       <c r="L7" s="5" t="inlineStr">
         <is>
-          <t>130/336 (66+64)</t>
-        </is>
-      </c>
-      <c r="M7" s="5" t="inlineStr">
-        <is>
-          <t>50m wall (40.5m Phase A+B + 9.6m Phase C)</t>
-        </is>
-      </c>
-      <c r="N7" s="4" t="n">
-        <v>1.3431</v>
+          <t>362 chunks (68+64+90+140) + 15 translate (4+4+6+9) ~177m wall (50m earlier +12.4m A+95m B+20m C)</t>
+        </is>
+      </c>
+      <c r="M7" s="5" t="n">
+        <v>3.835</v>
+      </c>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t>4/4 DONE 18+18+28+32 ch 68+64+90+140 no ==== Ch 18/18 28/28 32/32; Kazhar 0 anomalies clean, Kannappa 2 tails fixed 128 0-&gt;2312 147 7-&gt;774 re-merged 435893; English chunked 4+4+6+9 sequential 60K stop; Day6 heritage 96/96 DONE</t>
+        </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>Partial — 2/4 Done, 251/261 tails 0 flagged, 246 HUGE fixed, 493 fixed, 2-parallel, download retry 120s 3x</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">

</xml_diff>

<commit_message>
fix(periapuranam): Day6 tracker Day 6 sheet Kazhar 28/28 90ch + Kannappa 32/32 140ch Done — fix To be done, align DayWise_Plan 3.67
</commit_message>
<xml_diff>
--- a/periapuranam/day_wise_plan.xlsx
+++ b/periapuranam/day_wise_plan.xlsx
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="M7" s="5" t="n">
-        <v>3.835</v>
+        <v>3.6721</v>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
@@ -8332,24 +8332,44 @@
       </c>
       <c r="I5" s="23" t="inlineStr">
         <is>
-          <t>To be done</t>
-        </is>
-      </c>
-      <c r="J5" s="21" t="inlineStr"/>
-      <c r="K5" s="21" t="inlineStr"/>
-      <c r="L5" s="22" t="inlineStr"/>
-      <c r="M5" s="22" t="inlineStr"/>
-      <c r="N5" s="22" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J5" s="21" t="inlineStr">
+        <is>
+          <t>28/28</t>
+        </is>
+      </c>
+      <c r="K5" s="21" t="n">
+        <v>90</v>
+      </c>
+      <c r="L5" s="22" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="M5" s="22" t="n">
+        <v>0.2021</v>
+      </c>
+      <c r="N5" s="22" t="n">
+        <v>0.9221</v>
+      </c>
       <c r="O5" s="21" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P5" s="22" t="inlineStr"/>
-      <c r="Q5" s="22" t="inlineStr"/>
+      <c r="P5" s="22" t="inlineStr">
+        <is>
+          <t>0 anomalies; Phase A 28/28 12.4m 2-parallel; Phase B 90ch 95m 4-parallel resume (Budget 403 monthly fix); 8 empty mp3 skipped (395B)</t>
+        </is>
+      </c>
+      <c r="Q5" s="22" t="inlineStr">
+        <is>
+          <t>12.4m A + 95m B wall 287K Tamil 789KB 28ch no ====; English chunked 6x60K 292K bilingual 1081K 8.1m sequential</t>
+        </is>
+      </c>
       <c r="R5" s="22" t="inlineStr">
         <is>
-          <t>periapuranam/output/kazharitrarivar_nayanar/tamil_real/kazharitrarivar_nayanar_tamil.txt ; kazharitrarivar_nayanar_english.txt</t>
+          <t>periapuranam/output/day-06/kazharitrarivar_nayanar/tamil_real/kazharitrarivar_nayanar_tamil.txt ; english_real/6 chunks; kazharitrarivar_nayanar_english.txt</t>
         </is>
       </c>
     </row>
@@ -8390,24 +8410,44 @@
       </c>
       <c r="I6" s="23" t="inlineStr">
         <is>
-          <t>To be done</t>
-        </is>
-      </c>
-      <c r="J6" s="21" t="inlineStr"/>
-      <c r="K6" s="21" t="inlineStr"/>
-      <c r="L6" s="22" t="inlineStr"/>
-      <c r="M6" s="22" t="inlineStr"/>
-      <c r="N6" s="22" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J6" s="21" t="inlineStr">
+        <is>
+          <t>32/32</t>
+        </is>
+      </c>
+      <c r="K6" s="21" t="n">
+        <v>140</v>
+      </c>
+      <c r="L6" s="22" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="M6" s="22" t="n">
+        <v>0.2869</v>
+      </c>
+      <c r="N6" s="22" t="n">
+        <v>1.4069</v>
+      </c>
       <c r="O6" s="21" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P6" s="22" t="inlineStr"/>
-      <c r="Q6" s="22" t="inlineStr"/>
+      <c r="P6" s="22" t="inlineStr">
+        <is>
+          <t>2 tails fixed 128 EMPTY 0-&gt;2312 dur225 147 TINY 7-&gt;774 dur62 re-merged 435893; Phase B 95m 4-parallel resume Budget 403</t>
+        </is>
+      </c>
+      <c r="Q6" s="22" t="inlineStr">
+        <is>
+          <t>12.4m A + 95m B wall 435K Tamil 1193KB 32ch no ==== anomalies 0 after fix; English chunked 9x60K 421K bilingual 1615K 11.8m sequential; arrow cp1252 fix</t>
+        </is>
+      </c>
       <c r="R6" s="22" t="inlineStr">
         <is>
-          <t>periapuranam/output/kannappa_nayanar/tamil_real/kannappa_nayanar_tamil.txt ; kannappa_nayanar_english.txt</t>
+          <t>periapuranam/output/day-06/kannappa_nayanar/tamil_real/kannappa_nayanar_tamil.txt ; english_real/9 chunks; kannappa_nayanar_english.txt</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(periapuranam): Day7 partial Tiruk Kurippu Tonda 36F 129ch 399K Tamil 389K English 8ch
- Phase A 36/36 8m 9-17MB 608-1121s ffprobe skip
- Phase B 129ch ~55m 22s/ch +2s throttle cost Tamil 1.107: 225 chunk03 1.37s HUGE 43636 finish:length 12000 repeat loop beyond 901s valid audio removed 54184->10546 story 443178->399540 backup Huge, 235 TINY 17 Thiruchitrambalam accepted valid, ch17 retrans 3ch stable diff <50
- Phase C 8x60K stop ~12m cost 0.267 52585+49459+59349+54166+54165+51526+50030+18670 =389965 finish:stop no ==== Ch36 bilingual 1486KB
- Verification no ==== Ch36==36 files finish:stop instrumentation anomalies 0
- Tracker Day7 Tiruk Done 36/36 129ch 1.107+0.267=1.374 No, Sundarar Deferred per owner 2026-09-18, DayWise_Plan Row7 Partial 36/72 wall ~75m
- Runner periapuranam/run_tiruk_kurippu_tonda_nayanar.py DAY day-07 slug match

Selective backup 63 files output/day-07/tiruk_kurippu_tonda_nayanar (ignore audio chunk txt)
</commit_message>
<xml_diff>
--- a/periapuranam/day_wise_plan.xlsx
+++ b/periapuranam/day_wise_plan.xlsx
@@ -41,9 +41,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
+    <numFmt numFmtId="166" formatCode="0.000"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -279,7 +280,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -394,6 +395,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1300,16 +1304,34 @@
           <t>$2.43</t>
         </is>
       </c>
-      <c r="J8" s="5" t="inlineStr"/>
-      <c r="K8" s="5" t="inlineStr"/>
-      <c r="L8" s="5" t="inlineStr"/>
-      <c r="M8" s="5" t="inlineStr"/>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>36/72 (1/2 stories)</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>129ch + 8 translate ~75m wall (8m A +55m B +12m C)</t>
+        </is>
+      </c>
+      <c r="M8" s="41" t="n">
+        <v>1.3742</v>
+      </c>
       <c r="N8" s="4" t="inlineStr">
         <is>
-          <t>36-file stories: check Chapter count Sundarar discuss separately</t>
-        </is>
-      </c>
-      <c r="O8" s="2" t="inlineStr"/>
+          <t>Tiruk Kurippu 36/36 DONE 129ch 399540 Tamil 389965 English no ==== Ch36 1 HUGE fixed 225-&gt;10546; Sundarar DEFERRED per owner</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="52" customHeight="1">
       <c r="A9" s="2" t="n">
@@ -1706,7 +1728,7 @@
       </c>
       <c r="I3" s="23" t="inlineStr">
         <is>
-          <t>To be done</t>
+          <t>Deferred</t>
         </is>
       </c>
       <c r="J3" s="21" t="inlineStr"/>
@@ -1719,8 +1741,16 @@
           <t>No</t>
         </is>
       </c>
-      <c r="P3" s="22" t="inlineStr"/>
-      <c r="Q3" s="22" t="inlineStr"/>
+      <c r="P3" s="22" t="inlineStr">
+        <is>
+          <t>DEFERRED until further notice per owner 2026-09-18</t>
+        </is>
+      </c>
+      <c r="Q3" s="22" t="inlineStr">
+        <is>
+          <t>Sundarar 36 files deferred — awaiting sequence determination for remaining files beyond day-07</t>
+        </is>
+      </c>
       <c r="R3" s="22" t="inlineStr">
         <is>
           <t>periapuranam/output/sundarar/tamil_real/sundarar_tamil.txt ; sundarar_english.txt</t>
@@ -1764,24 +1794,44 @@
       </c>
       <c r="I4" s="23" t="inlineStr">
         <is>
-          <t>To be done</t>
-        </is>
-      </c>
-      <c r="J4" s="21" t="inlineStr"/>
-      <c r="K4" s="21" t="inlineStr"/>
-      <c r="L4" s="22" t="inlineStr"/>
-      <c r="M4" s="22" t="inlineStr"/>
-      <c r="N4" s="22" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J4" s="21" t="inlineStr">
+        <is>
+          <t>36/36</t>
+        </is>
+      </c>
+      <c r="K4" s="21" t="n">
+        <v>129</v>
+      </c>
+      <c r="L4" s="44" t="n">
+        <v>1.107</v>
+      </c>
+      <c r="M4" s="44" t="n">
+        <v>0.267</v>
+      </c>
+      <c r="N4" s="44" t="n">
+        <v>1.374</v>
+      </c>
       <c r="O4" s="21" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="P4" s="22" t="inlineStr"/>
-      <c r="Q4" s="22" t="inlineStr"/>
+      <c r="P4" s="22" t="inlineStr">
+        <is>
+          <t>1 HUGE 225c03 43k 1s hallucination beyond valid audio 901s removed re-merged 10546 vs 54184 (cost 0.029); 1 TINY 235c03 17 accepted valid Thiruchitrambalam; ch17 retrans diff &lt;50 stable</t>
+        </is>
+      </c>
+      <c r="Q4" s="22" t="inlineStr">
+        <is>
+          <t>3-phase A 36/36 8m B 129ch 55m C 8ch 12m wall ~75m 399540 Tamil 1096KB 389965 English 390KB bilingual 1486KB no ==== Ch36; ch17 fixed tail silence; english chunked 8x60K stop (3 cached +5 new)</t>
+        </is>
+      </c>
       <c r="R4" s="22" t="inlineStr">
         <is>
-          <t>periapuranam/output/tiruk_kurippu_tonda_nayanar/tamil_real/tiruk_kurippu_tonda_nayanar_tamil.txt ; tiruk_kurippu_tonda_nayanar_english.txt</t>
+          <t>periapuranam/output/day-07/tiruk_kurippu_tonda_nayanar/tamil_real/tiruk_kurippu_tonda_nayanar_tamil.txt ; tiruk_kurippu_tonda_nayanar_english.txt ; english_real/8 chunks</t>
         </is>
       </c>
     </row>

</xml_diff>